<commit_message>
Rebuild BL template (100KB from 660MB), rewrite exportBLExcel with direct cell writes
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5cbf0556e688d176/VScode/Gestion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahb\Desktop\Thécol\Finances\Livraison et facturation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{3DAFF786-19DC-46E3-9842-2A4D9660460B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0934A997-E35F-4BFA-9FB3-9F485C805EC8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF0E999-4ECE-4970-AD15-5307EE881E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{C5804516-DE8A-4579-A9F8-8DDE14F0BC4E}"/>
+    <workbookView xWindow="3660" yWindow="2085" windowWidth="28800" windowHeight="15345" xr2:uid="{C5804516-DE8A-4579-A9F8-8DDE14F0BC4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulletin de livraison" sheetId="1" r:id="rId1"/>
@@ -27,36 +27,16 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="210">
   <si>
     <t>local – artisanal – saveurs originales</t>
   </si>
@@ -79,6 +59,9 @@
     <t>Arôme</t>
   </si>
   <si>
+    <t>Liste arômes</t>
+  </si>
+  <si>
     <t>Poire à Botzi</t>
   </si>
   <si>
@@ -97,6 +80,9 @@
     <t>Edition Noël</t>
   </si>
   <si>
+    <t>Liste Formats</t>
+  </si>
+  <si>
     <t>25 cl</t>
   </si>
   <si>
@@ -106,6 +92,189 @@
     <t>100 cl</t>
   </si>
   <si>
+    <t>Adresse</t>
+  </si>
+  <si>
+    <t>Société</t>
+  </si>
+  <si>
+    <t>Tarifs</t>
+  </si>
+  <si>
+    <t>1.2.3 Bocal</t>
+  </si>
+  <si>
+    <t>Route de Fribourg 7a</t>
+  </si>
+  <si>
+    <t>Liste Tarifs</t>
+  </si>
+  <si>
+    <t>Distributeur</t>
+  </si>
+  <si>
+    <t>Privé</t>
+  </si>
+  <si>
+    <t>Spécial</t>
+  </si>
+  <si>
+    <t>Au Bon Moment</t>
+  </si>
+  <si>
+    <t>Route de Fribourg 17</t>
+  </si>
+  <si>
+    <t>Audiopur</t>
+  </si>
+  <si>
+    <t>Rue de Lausanne 60</t>
+  </si>
+  <si>
+    <t>La ferme Planchy</t>
+  </si>
+  <si>
+    <t>Rue du Rosé 61</t>
+  </si>
+  <si>
+    <t>La grande Planche 2</t>
+  </si>
+  <si>
+    <t>Fribourg Natation</t>
+  </si>
+  <si>
+    <t>L'ART'isan Pâtissier</t>
+  </si>
+  <si>
+    <t>Route de Fribourg 12</t>
+  </si>
+  <si>
+    <t>La Vracrie</t>
+  </si>
+  <si>
+    <t>Route Principale 90</t>
+  </si>
+  <si>
+    <t>Les Bièrosophes Sàrl</t>
+  </si>
+  <si>
+    <t>Rue du Valentin 7</t>
+  </si>
+  <si>
+    <t>L'épicerie Papiy Sàrl</t>
+  </si>
+  <si>
+    <t>Ruelle Thomas 21</t>
+  </si>
+  <si>
+    <t>Piccand Vins &amp; Boissons</t>
+  </si>
+  <si>
+    <t>Route des Grandseys 81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técole </t>
+  </si>
+  <si>
+    <t>Rue de l'église 75</t>
+  </si>
+  <si>
+    <t>Terre d'Elles</t>
+  </si>
+  <si>
+    <t>Route du Barrage 21</t>
+  </si>
+  <si>
+    <t>Terroir Fribourg</t>
+  </si>
+  <si>
+    <t>Route de Chantemerie 41</t>
+  </si>
+  <si>
+    <t>1784 Courtepin</t>
+  </si>
+  <si>
+    <t>1723 Marly</t>
+  </si>
+  <si>
+    <t>1700 Fribourg</t>
+  </si>
+  <si>
+    <t>1630 Bulle</t>
+  </si>
+  <si>
+    <t>1733 Treyvaux</t>
+  </si>
+  <si>
+    <t>1746 Prez-vers-Noréaz</t>
+  </si>
+  <si>
+    <t>1400 Yverdon-les-Bains</t>
+  </si>
+  <si>
+    <t>1618 Châtel-St-Denis</t>
+  </si>
+  <si>
+    <t>1564 Domdidier</t>
+  </si>
+  <si>
+    <t>1680 Romont</t>
+  </si>
+  <si>
+    <t>1763 Granges-Paccot</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NPA &amp; Localité</t>
+  </si>
+  <si>
+    <t>Prénom &amp; Nom</t>
+  </si>
+  <si>
+    <t>Nathalie Oberson</t>
+  </si>
+  <si>
+    <t>Céline Jeanbourquin</t>
+  </si>
+  <si>
+    <t>Michael Deforné</t>
+  </si>
+  <si>
+    <t>Elisa Crausaz</t>
+  </si>
+  <si>
+    <t>Christian Hejda</t>
+  </si>
+  <si>
+    <t>Nicolas Rouiller</t>
+  </si>
+  <si>
+    <t>Alain Kaehr</t>
+  </si>
+  <si>
+    <t>Laure Niquille Rahmann</t>
+  </si>
+  <si>
+    <t>Emmanuelle Piccand</t>
+  </si>
+  <si>
+    <t>Claude Oberson</t>
+  </si>
+  <si>
+    <t>Caroline Masotti</t>
+  </si>
+  <si>
+    <t>Yannick Etter</t>
+  </si>
+  <si>
+    <t>Véronique Beaud</t>
+  </si>
+  <si>
+    <t>Brodard Christiane</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>Livré : "ancienne caisse verte" IFCO</t>
   </si>
   <si>
@@ -118,6 +287,27 @@
     <t>Retour : "nouvelle caisse noire" IFCO</t>
   </si>
   <si>
+    <t>Mode facturation favorit</t>
+  </si>
+  <si>
+    <t>Mode facturation</t>
+  </si>
+  <si>
+    <t>E-Mail</t>
+  </si>
+  <si>
+    <t>Envoi postal</t>
+  </si>
+  <si>
+    <t>Coordonnées relatives</t>
+  </si>
+  <si>
+    <t>info@aubonmoment.ch</t>
+  </si>
+  <si>
+    <t>info@terredelles.ch</t>
+  </si>
+  <si>
     <t>ThéCol - Thé Froid Artisanal</t>
   </si>
   <si>
@@ -130,6 +320,9 @@
     <t>Autre :</t>
   </si>
   <si>
+    <t>michael@audiopur.ch</t>
+  </si>
+  <si>
     <t>Dégustation Su.</t>
   </si>
   <si>
@@ -142,17 +335,347 @@
     <t xml:space="preserve">À </t>
   </si>
   <si>
+    <t>contact@123bocal.ch</t>
+  </si>
+  <si>
+    <t>Escape and Fun</t>
+  </si>
+  <si>
+    <t>Coralie Boss</t>
+  </si>
+  <si>
+    <t>Route de Portalban 11</t>
+  </si>
+  <si>
+    <t>1567 Delley</t>
+  </si>
+  <si>
+    <t>boss.coralie@gmail.com</t>
+  </si>
+  <si>
+    <t>1788 Praz Vully</t>
+  </si>
+  <si>
+    <t>info@art-isan.ch</t>
+  </si>
+  <si>
+    <t>vero.beaud@hotmail.com</t>
+  </si>
+  <si>
+    <t>info@lesbierosophes.ch</t>
+  </si>
+  <si>
+    <t>yannick.etter@terroir-fribourg.ch</t>
+  </si>
+  <si>
+    <t>emmanuellepiccand@gmail.com</t>
+  </si>
+  <si>
+    <t>laureniquille@gmail.com</t>
+  </si>
+  <si>
+    <t>Fribourg Cybersecurity seminar</t>
+  </si>
+  <si>
+    <t>HEIA-FR Michael Mäder</t>
+  </si>
+  <si>
+    <t>Bd de Pérolles 80</t>
+  </si>
+  <si>
+    <t>1700, Fribourg</t>
+  </si>
+  <si>
+    <t>sur place à la livraison</t>
+  </si>
+  <si>
+    <t>cricrihejda@gmail.com</t>
+  </si>
+  <si>
+    <t>Rue du Village 10</t>
+  </si>
+  <si>
+    <t>1034, Bousens</t>
+  </si>
+  <si>
+    <t>Bastien Jaccaud</t>
+  </si>
+  <si>
+    <t>Le Chalet de Boussens</t>
+  </si>
+  <si>
+    <t>WhatsApp : 079 381 59 87</t>
+  </si>
+  <si>
+    <t>Stéphanie Derron</t>
+  </si>
+  <si>
+    <t>derron.stephanie@gmail.com</t>
+  </si>
+  <si>
+    <t>Ia Vracrie</t>
+  </si>
+  <si>
+    <t>Angéloz Mode</t>
+  </si>
+  <si>
+    <t>Jonathan.Collaud@angeloz-mode.ch</t>
+  </si>
+  <si>
+    <t>Centre la Tour</t>
+  </si>
+  <si>
+    <t>Route de Pra-Riond 2</t>
+  </si>
+  <si>
+    <t>1635 La Tour-de-Trême</t>
+  </si>
+  <si>
+    <t>Café de la Marionnette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ines Haymoz </t>
+  </si>
+  <si>
+    <t>Derrière-les-Jardins 2</t>
+  </si>
+  <si>
+    <t>camille.marion@hotmail.com</t>
+  </si>
+  <si>
+    <t>Camille Marion</t>
+  </si>
+  <si>
+    <t>Festival du Film Vert de la Broye</t>
+  </si>
+  <si>
+    <t>Commission Subsistance</t>
+  </si>
+  <si>
+    <t>1544 Gletterens</t>
+  </si>
+  <si>
+    <t>Pierrick Jay</t>
+  </si>
+  <si>
+    <t>Sherlock Club, Patricia Ferltrin</t>
+  </si>
+  <si>
+    <t>Grand-Rue 96</t>
+  </si>
+  <si>
+    <t>1110 Morges</t>
+  </si>
+  <si>
+    <t>contact@sherlock-events.ch</t>
+  </si>
+  <si>
+    <t>ES Belfaux</t>
+  </si>
+  <si>
+    <t>Case postale 14</t>
+  </si>
+  <si>
+    <t>1782 Belfaux</t>
+  </si>
+  <si>
+    <t>Caroline Benoit</t>
+  </si>
+  <si>
+    <t>info@esbelfaux.ch</t>
+  </si>
+  <si>
+    <t>Au Petit Marché</t>
+  </si>
+  <si>
+    <t>Dominique Weislo</t>
+  </si>
+  <si>
+    <t>Rue de la Neuveville 68</t>
+  </si>
+  <si>
+    <t>Mérillat SA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabrielle Kocher </t>
+  </si>
+  <si>
+    <t>Les Cornette 6</t>
+  </si>
+  <si>
+    <t>2735 Malleray BE</t>
+  </si>
+  <si>
+    <t>gabrielle@merillatsa.ch</t>
+  </si>
+  <si>
+    <t>L'Esprit du Fruit</t>
+  </si>
+  <si>
+    <t>Valentin Blondel</t>
+  </si>
+  <si>
+    <t>Rue d'Yverdon 19</t>
+  </si>
+  <si>
+    <t>1023 Crissier</t>
+  </si>
+  <si>
+    <t>commandes@mblondel.ch</t>
+  </si>
+  <si>
+    <t>L'Antre d'Eux</t>
+  </si>
+  <si>
+    <t>Aurore Borrat-Besson</t>
+  </si>
+  <si>
+    <t>Rte de Champoussin 22</t>
+  </si>
+  <si>
+    <t>1873 Champoussin</t>
+  </si>
+  <si>
+    <t>lantredeuxchampoussin@gmail.com</t>
+  </si>
+  <si>
+    <t>Didier Ecoffey</t>
+  </si>
+  <si>
+    <t>Grand-Rue 4</t>
+  </si>
+  <si>
+    <t>Boulangerie Didier Ecoffey</t>
+  </si>
+  <si>
+    <t>boulangerie.ecoffey@bluewin.ch</t>
+  </si>
+  <si>
+    <t>Fromagerie de Rossens</t>
+  </si>
+  <si>
+    <t>Vincent Guillet</t>
+  </si>
+  <si>
+    <t>Route du Barrage 100</t>
+  </si>
+  <si>
+    <t>1728 Rossens</t>
+  </si>
+  <si>
+    <t>fromagerieguillet@bluewin.ch</t>
+  </si>
+  <si>
+    <t>La ferme du Ferrage</t>
+  </si>
+  <si>
+    <t>Aurélie Pittet</t>
+  </si>
+  <si>
+    <t>Route du ferrage 21</t>
+  </si>
+  <si>
+    <t>1695 Rueyres-St-Laurent</t>
+  </si>
+  <si>
+    <t>lafermeduferrage@bluewin.ch</t>
+  </si>
+  <si>
+    <t>Au Bocal du Coin</t>
+  </si>
+  <si>
+    <t>Stéphanie Caille</t>
+  </si>
+  <si>
+    <t>Grand-Rue 26</t>
+  </si>
+  <si>
+    <t>aubocalducoin@hotmail.com</t>
+  </si>
+  <si>
+    <t>Fromagerie de Villaz-St-Pierre</t>
+  </si>
+  <si>
+    <t>Vincent Rohrbasser</t>
+  </si>
+  <si>
+    <t>Route de Fuyens 14</t>
+  </si>
+  <si>
+    <t>1690 Villaz-St.-Pierre</t>
+  </si>
+  <si>
+    <t>fromagerievillaz@outlook.com</t>
+  </si>
+  <si>
+    <t>Fromagerie de Ponthaux</t>
+  </si>
+  <si>
+    <t>Aline Ponti</t>
+  </si>
+  <si>
+    <t>Au Village 13</t>
+  </si>
+  <si>
+    <t>1772 Ponthaux</t>
+  </si>
+  <si>
+    <t>aline_ponti@hotmail.com</t>
+  </si>
+  <si>
+    <t>Angelica Verani</t>
+  </si>
+  <si>
+    <t>Bar Gelateria Verani</t>
+  </si>
+  <si>
+    <t>Rue de la Neuveville 52</t>
+  </si>
+  <si>
+    <t>angelica.verani@xs4all.nl</t>
+  </si>
+  <si>
+    <t>Assemblage</t>
+  </si>
+  <si>
+    <t>Gisèle Maudua-Gachet</t>
+  </si>
+  <si>
+    <t>Pl. de l'Ancienne Papetterie 4</t>
+  </si>
+  <si>
+    <t>mathilde.devaud@akdagsa.ch</t>
+  </si>
+  <si>
     <t>Coing</t>
   </si>
   <si>
     <t>Facturation :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grangeneuve </t>
+  </si>
+  <si>
+    <t>Gilles Genoud</t>
+  </si>
+  <si>
+    <t>Route de Grangeneuve 19</t>
+  </si>
+  <si>
+    <t>1725 Posieux</t>
+  </si>
+  <si>
+    <t>gilles.genoud@fr.ch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="10">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+  </numFmts>
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,6 +731,26 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -329,10 +872,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -346,6 +890,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -384,6 +932,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -391,21 +940,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;CHF&quot;"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -794,72 +1365,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE0EAD78-21B9-453B-AABA-02EE8646C4F8}" name="Tableau1" displayName="Tableau1" ref="A14:D44" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE0EAD78-21B9-453B-AABA-02EE8646C4F8}" name="Tableau1" displayName="Tableau1" ref="A14:D44" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A14:D44" xr:uid="{DE0EAD78-21B9-453B-AABA-02EE8646C4F8}">
     <filterColumn colId="0">
       <filters blank="1">
@@ -871,12 +1378,12 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1A477314-2E09-4C98-BAC6-896516FACBCF}" name="QTT" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{38558BE9-82AC-43AB-A07D-B067A83EA99E}" name="Description" dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{1A477314-2E09-4C98-BAC6-896516FACBCF}" name="QTT" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{38558BE9-82AC-43AB-A07D-B067A83EA99E}" name="Description" dataDxfId="7">
       <calculatedColumnFormula>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8422D6DD-456B-478D-A22C-DE624EDE619C}" name="Arôme" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{975D51B1-3BEB-45A8-9486-4C2BEDCCBA24}" name="Format" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{8422D6DD-456B-478D-A22C-DE624EDE619C}" name="Arôme" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{975D51B1-3BEB-45A8-9486-4C2BEDCCBA24}" name="Format" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1197,622 +1704,6 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
-  <dimension ref="A2:F61"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="6.5703125" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="5.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:6" ht="22.5" customHeight="1">
-      <c r="F2" s="7"/>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="E4" s="18"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="E5" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4">
-        <f ca="1">TODAY()</f>
-        <v>46108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.5">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="E7" s="18"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="E9" s="5"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="E10" s="5"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="12" spans="1:6" ht="7.5" customHeight="1"/>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" hidden="1">
-      <c r="A15" s="24">
-        <v>0</v>
-      </c>
-      <c r="B15" s="19" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" hidden="1">
-      <c r="A16" s="25">
-        <v>0</v>
-      </c>
-      <c r="B16" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="25"/>
-      <c r="B17" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="12"/>
-    </row>
-    <row r="18" spans="1:4" hidden="1">
-      <c r="A18" s="25">
-        <v>0</v>
-      </c>
-      <c r="B18" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" hidden="1">
-      <c r="A19" s="25">
-        <v>0</v>
-      </c>
-      <c r="B19" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" hidden="1">
-      <c r="A20" s="25">
-        <v>0</v>
-      </c>
-      <c r="B20" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" hidden="1">
-      <c r="A21" s="25">
-        <v>0</v>
-      </c>
-      <c r="B21" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" hidden="1">
-      <c r="A22" s="25">
-        <v>0</v>
-      </c>
-      <c r="B22" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" hidden="1">
-      <c r="A23" s="25">
-        <v>0</v>
-      </c>
-      <c r="B23" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" hidden="1">
-      <c r="A24" s="25">
-        <v>0</v>
-      </c>
-      <c r="B24" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" hidden="1">
-      <c r="A25" s="25">
-        <v>0</v>
-      </c>
-      <c r="B25" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" hidden="1">
-      <c r="A26" s="25">
-        <v>0</v>
-      </c>
-      <c r="B26" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" hidden="1">
-      <c r="A27" s="25">
-        <v>0</v>
-      </c>
-      <c r="B27" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" hidden="1">
-      <c r="A28" s="25">
-        <v>0</v>
-      </c>
-      <c r="B28" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="25"/>
-      <c r="B29" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="13"/>
-    </row>
-    <row r="30" spans="1:4" hidden="1">
-      <c r="A30" s="25">
-        <v>0</v>
-      </c>
-      <c r="B30" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" hidden="1">
-      <c r="A31" s="25">
-        <v>0</v>
-      </c>
-      <c r="B31" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="25"/>
-      <c r="B32" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C32" s="14"/>
-      <c r="D32" s="13"/>
-    </row>
-    <row r="33" spans="1:5" hidden="1">
-      <c r="A33" s="25">
-        <v>0</v>
-      </c>
-      <c r="B33" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" hidden="1">
-      <c r="A34" s="25">
-        <v>0</v>
-      </c>
-      <c r="B34" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="25"/>
-      <c r="B35" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="13"/>
-    </row>
-    <row r="36" spans="1:5" hidden="1">
-      <c r="A36" s="25">
-        <v>0</v>
-      </c>
-      <c r="B36" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" hidden="1">
-      <c r="A37" s="25">
-        <v>0</v>
-      </c>
-      <c r="B37" s="8" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" hidden="1">
-      <c r="A38" s="25">
-        <v>0</v>
-      </c>
-      <c r="B38" s="22" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A39" s="25"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="9"/>
-    </row>
-    <row r="40" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A40" s="27"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-    </row>
-    <row r="41" spans="1:5" ht="2.25" hidden="1" customHeight="1">
-      <c r="A41" s="25">
-        <v>0</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="28"/>
-    </row>
-    <row r="42" spans="1:5" hidden="1">
-      <c r="A42" s="25">
-        <v>0</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C42" s="10"/>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" spans="1:5" hidden="1">
-      <c r="A43" s="25">
-        <v>0</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:5" ht="15" customHeight="1">
-      <c r="B46" s="17"/>
-      <c r="C46" s="16"/>
-      <c r="D46" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="2"/>
-      <c r="E47" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="15" customHeight="1" thickBot="1">
-      <c r="A48" s="29"/>
-      <c r="B48" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="2"/>
-      <c r="E48" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="15" customHeight="1" thickBot="1">
-      <c r="A49" s="29"/>
-      <c r="B49" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="16"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="31" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="15" customHeight="1" thickBot="1">
-      <c r="A50" s="29"/>
-      <c r="B50" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" s="16"/>
-      <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="1:6" ht="15.75" thickBot="1">
-      <c r="A51" s="30"/>
-      <c r="B51" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C51" s="16"/>
-      <c r="D51" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51" s="32" t="e">
-        <f>VLOOKUP(F7,#REF!,10,FALSE)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" spans="1:6" ht="28.5" customHeight="1">
-      <c r="B52" s="26"/>
-      <c r="C52" s="16"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" spans="1:6">
-      <c r="B53" s="16"/>
-      <c r="C53" s="16"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-    </row>
-    <row r="54" spans="1:6" ht="21">
-      <c r="A54" s="6">
-        <f>F7</f>
-        <v>0</v>
-      </c>
-      <c r="B54" s="16"/>
-      <c r="C54" s="16"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" spans="1:6" ht="42" customHeight="1">
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-    </row>
-    <row r="56" spans="1:6" ht="21">
-      <c r="A56" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B56" s="6"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="1:6" ht="51" customHeight="1">
-      <c r="D57" s="33" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="E57" s="33"/>
-      <c r="F57" s="33"/>
-    </row>
-    <row r="58" spans="1:6">
-      <c r="B58" s="33"/>
-      <c r="D58" s="33"/>
-      <c r="E58" s="33"/>
-      <c r="F58" s="33"/>
-    </row>
-    <row r="59" spans="1:6">
-      <c r="B59" s="33"/>
-      <c r="D59" s="33"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
-    </row>
-    <row r="60" spans="1:6">
-      <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="1:6">
-      <c r="D61" s="2"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="D57:F59"/>
-  </mergeCells>
-  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
-  </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F88F0296-B037-4558-8BF3-BF1788835FEC}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>F7</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F91DE666-C1EC-46FF-BFAC-77ABE88F7950}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>C15:C38</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B9B91086-C40D-46C4-8549-1E3A0C7DF361}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>D15:D38</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
-</worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac xr xr2 xr3" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}"><dimension ref="A2:F61"/><sheetFormatPr baseColWidth="10" defaultRowHeight="15"/><cols><col min="1" max="1" width="6.5703125" customWidth="1"/><col min="2" max="2" width="23.7109375" customWidth="1"/><col min="3" max="3" width="15" customWidth="1"/><col min="4" max="4" width="5.7109375" customWidth="1"/><col min="5" max="5" width="11.28515625" customWidth="1"/><col min="6" max="6" width="16.85546875" customWidth="1"/></cols><sheetData><row r="2" spans="1:6" ht="22.5" customHeight="1"><c r="F2" s="7"/></row><row r="3" spans="1:6"><c r="F3" s="2"/></row><row r="4" spans="1:6"><c r="E4" s="20"/><c r="F4" s="4"/></row><row r="5" spans="1:6"><c r="E5" s="20" t="s"><v>1</v></c><c r="F5" s="4"></c></row><row r="6" spans="1:6" ht="16.5"><c r="A6" s="1" t="s"><v>0</v></c><c r="B6" s="1"/><c r="E6" s="5"/><c r="F6" s="5"/></row><row r="7" spans="1:6"><c r="E7" s="20"/><c r="F7" s="3"></c></row><row r="8" spans="1:6"><c r="E8" s="3"/><c r="F8" s="3"></c></row><row r="9" spans="1:6"><c r="E9" s="5"/><c r="F9" s="3"></c></row><row r="10" spans="1:6"><c r="E10" s="5"/><c r="F10" s="3"></c></row><row r="12" spans="1:6" ht="7.5" customHeight="1"/><row r="14" spans="1:6"><c r="A14" s="5" t="s"><v>3</v></c><c r="B14" s="5" t="s"><v>4</v></c><c r="C14" s="25" t="s"><v>6</v></c><c r="D14" s="25" t="s"><v>5</v></c></row><row r="15" spans="1:6" hidden="1"><c r="A15" s="26"><v>0</v></c><c r="B15" s="21" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C15" s="22" t="s"><v>8</v></c><c r="D15" s="23" t="s"><v>15</v></c></row><row r="16" spans="1:6" hidden="1"><c r="A16" s="27"><v>0</v></c><c r="B16" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C16" s="16" t="s"><v>8</v></c><c r="D16" s="14" t="s"><v>16</v></c></row><row r="17" spans="1:4"><c r="A17" s="27"><v>18</v></c><c r="B17" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C17" s="16" t="s"><v>8</v></c><c r="D17" s="14" t="s"><v>17</v></c></row><row r="18" spans="1:4" hidden="1"><c r="A18" s="27"><v>0</v></c><c r="B18" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C18" s="16" t="s"><v>11</v></c><c r="D18" s="14" t="s"><v>15</v></c></row><row r="19" spans="1:4" hidden="1"><c r="A19" s="27"><v>0</v></c><c r="B19" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C19" s="16" t="s"><v>11</v></c><c r="D19" s="14" t="s"><v>16</v></c></row><row r="20" spans="1:4" hidden="1"><c r="A20" s="27"><v>0</v></c><c r="B20" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C20" s="16" t="s"><v>11</v></c><c r="D20" s="14" t="s"><v>17</v></c></row><row r="21" spans="1:4" hidden="1"><c r="A21" s="27"><v>0</v></c><c r="B21" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C21" s="16" t="s"><v>9</v></c><c r="D21" s="14" t="s"><v>15</v></c></row><row r="22" spans="1:4" hidden="1"><c r="A22" s="27"><v>0</v></c><c r="B22" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C22" s="16" t="s"><v>9</v></c><c r="D22" s="14" t="s"><v>16</v></c></row><row r="23" spans="1:4" hidden="1"><c r="A23" s="27"><v>0</v></c><c r="B23" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C23" s="16" t="s"><v>9</v></c><c r="D23" s="14" t="s"><v>17</v></c></row><row r="24" spans="1:4" hidden="1"><c r="A24" s="27"><v>0</v></c><c r="B24" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C24" s="16" t="s"><v>10</v></c><c r="D24" s="14" t="s"><v>15</v></c></row><row r="25" spans="1:4" hidden="1"><c r="A25" s="27"><v>0</v></c><c r="B25" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C25" s="16" t="s"><v>10</v></c><c r="D25" s="14" t="s"><v>16</v></c></row><row r="26" spans="1:4" hidden="1"><c r="A26" s="27"><v>0</v></c><c r="B26" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C26" s="16" t="s"><v>10</v></c><c r="D26" s="14" t="s"><v>17</v></c></row><row r="27" spans="1:4" hidden="1"><c r="A27" s="27"><v>0</v></c><c r="B27" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C27" s="16" t="s"><v>12</v></c><c r="D27" s="14" t="s"><v>15</v></c></row><row r="28" spans="1:4" hidden="1"><c r="A28" s="27"><v>0</v></c><c r="B28" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C28" s="16" t="s"><v>12</v></c><c r="D28" s="14" t="s"><v>16</v></c></row><row r="29" spans="1:4"><c r="A29" s="27"><v>6</v></c><c r="B29" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C29" s="16" t="s"><v>12</v></c><c r="D29" s="15" t="s"><v>17</v></c></row><row r="30" spans="1:4" hidden="1"><c r="A30" s="27"><v>0</v></c><c r="B30" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C30" s="16" t="s"><v>91</v></c><c r="D30" s="15" t="s"><v>15</v></c></row><row r="31" spans="1:4" hidden="1"><c r="A31" s="27"><v>0</v></c><c r="B31" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C31" s="16" t="s"><v>91</v></c><c r="D31" s="15" t="s"><v>16</v></c></row><row r="32" spans="1:4"><c r="A32" s="27"><v>24</v></c><c r="B32" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C32" s="16" t="s"><v>91</v></c><c r="D32" s="15" t="s"><v>17</v></c></row><row r="33" spans="1:5" hidden="1"><c r="A33" s="27"><v>0</v></c><c r="B33" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C33" s="16" t="s"><v>203</v></c><c r="D33" s="15" t="s"><v>15</v></c></row><row r="34" spans="1:5" hidden="1"><c r="A34" s="27"><v>0</v></c><c r="B34" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C34" s="16" t="s"><v>203</v></c><c r="D34" s="15" t="s"><v>16</v></c></row><row r="35" spans="1:5"><c r="A35" s="27"><v>12</v></c><c r="B35" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C35" s="16" t="s"><v>203</v></c><c r="D35" s="15" t="s"><v>17</v></c></row><row r="36" spans="1:5" hidden="1"><c r="A36" s="27"><v>0</v></c><c r="B36" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C36" s="16" t="s"><v>13</v></c><c r="D36" s="14" t="s"><v>15</v></c></row><row r="37" spans="1:5" hidden="1"><c r="A37" s="27"><v>0</v></c><c r="B37" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C37" s="17" t="s"><v>13</v></c><c r="D37" s="14" t="s"><v>16</v></c></row><row r="38" spans="1:5" hidden="1"><c r="A38" s="27"><v>0</v></c><c r="B38" s="24" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C38" s="16" t="s"><v>13</v></c><c r="D38" s="15" t="s"><v>17</v></c></row><row r="39" spans="1:5" ht="14.25" customHeight="1"><c r="A39" s="27"/><c r="B39" s="10"/><c r="C39" s="13"/><c r="D39" s="11"/></row><row r="40" spans="1:5" ht="14.25" customHeight="1"><c r="A40" s="30"/><c r="B40" s="12"/><c r="C40" s="5"/><c r="D40" s="5"/></row><row r="41" spans="1:5" ht="2.25" hidden="1" customHeight="1"><c r="A41" s="27"><v>0</v></c><c r="B41" s="10" t="s"><v>92</v></c><c r="C41" s="11"/><c r="D41" s="31"/></row><row r="42" spans="1:5" hidden="1"><c r="A42" s="27"><v>0</v></c><c r="B42" s="10" t="s"><v>92</v></c><c r="C42" s="12"/><c r="D42" s="11"/></row><row r="43" spans="1:5" hidden="1"><c r="A43" s="27"><v>0</v></c><c r="B43" s="10" t="s"><v>90</v></c><c r="C43" s="13" t="s"><v>95</v></c><c r="D43" s="11" t="s"><v>17</v></c></row><row r="44" spans="1:5"><c r="A44" s="5"/><c r="B44" s="5" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C44" s="5"/><c r="D44" s="5"/></row><row r="45" spans="1:5" ht="14.25" customHeight="1"/><row r="46" spans="1:5" ht="15" customHeight="1"><c r="B46" s="19"/><c r="C46" s="18"/><c r="D46" t="s"><v>204</v></c></row><row r="47" spans="1:5" ht="15" customHeight="1" thickBot="1"><c r="B47" s="18"/><c r="C47" s="18"/><c r="D47" s="2"></c><c r="E47" t="s"><v>96</v></c></row><row r="48" spans="1:5" ht="15" customHeight="1" thickBot="1"><c r="A48" s="32"><v>0</v></c><c r="B48" s="28" t="s"><v>79</v></c><c r="C48" s="18"/><c r="D48" s="2"></c><c r="E48" t="s"><v>97</v></c></row><row r="49" spans="1:6" ht="15" customHeight="1" thickBot="1"><c r="A49" s="32"><v>3</v></c><c r="B49" s="28" t="s"><v>80</v></c><c r="C49" s="18"/><c r="D49" s="2"></c><c r="E49" s="36" t="s"><v>93</v></c></row><row r="50" spans="1:6" ht="15" customHeight="1" thickBot="1"><c r="A50" s="32"/><c r="B50" s="28" t="s"><v>81</v></c><c r="C50" s="18"/><c r="D50" s="2"/></row><row r="51" spans="1:6" ht="15.75" thickBot="1"><c r="A51" s="34"/><c r="B51" s="28" t="s"><v>82</v></c><c r="C51" s="18"/><c r="D51" t="s"><v>98</v></c><c r="E51" s="40"></c><c r="F51" s="2"/></row><row r="52" spans="1:6" ht="28.5" customHeight="1"><c r="B52" s="28"/><c r="C52" s="18"/><c r="E52" s="2"/><c r="F52" s="2"/></row><row r="53" spans="1:6"><c r="B53" s="18"/><c r="C53" s="18"/><c r="E53" s="2"/><c r="F53" s="2"/></row><row r="54" spans="1:6" ht="21"><c r="A54" s="6"></c><c r="B54" s="18"/><c r="C54" s="18"/><c r="E54" s="2"/><c r="F54" s="2"/></row><row r="55" spans="1:6" ht="42" customHeight="1"><c r="E55" s="2"/><c r="F55" s="2"/></row><row r="56" spans="1:6" ht="21"><c r="A56" s="6" t="s"><v>2</v></c><c r="B56" s="6"/><c r="E56" s="2"/><c r="F56" s="2"/></row><row r="57" spans="1:6" ht="51" customHeight="1"><c r="D57" s="38" t="e" vm="1"><v>#VALUE!</v></c><c r="E57" s="38"/><c r="F57" s="38"/></row><row r="58" spans="1:6"><c r="B58" s="38"/><c r="D58" s="38"/><c r="E58" s="38"/><c r="F58" s="38"/></row><row r="59" spans="1:6"><c r="B59" s="38"/><c r="D59" s="38"/><c r="E59" s="38"/><c r="F59" s="38"/></row><row r="60" spans="1:6"><c r="D60" s="2"/></row><row r="61" spans="1:6"><c r="D61" s="2"/></row></sheetData><mergeCells count="2"><mergeCell ref="B58:B59"/><mergeCell ref="D57:F59"/></mergeCells><pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/><pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/><drawing r:id="rId2"/><tableParts count="1"><tablePart r:id="rId3"/></tableParts><extLst><ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main"></x14:dataValidations></ext></extLst></worksheet>
 </file>
</xml_diff>

<commit_message>
Hotfix: rebuild bl_template.xlsx with proper XML parsing (fix corrupted extLst block)
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -1,35 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahb\Desktop\Thécol\Finances\Livraison et facturation\"/>
+      <ns2:absPath url="C:\Users\noahb\Desktop\Thécol\Finances\Livraison et facturation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF0E999-4ECE-4970-AD15-5307EE881E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF0E999-4ECE-4970-AD15-5307EE881E75}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2085" windowWidth="28800" windowHeight="15345" xr2:uid="{C5804516-DE8A-4579-A9F8-8DDE14F0BC4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulletin de livraison" sheetId="1" r:id="rId1"/>
+    <sheet name="Listes " sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns8:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns9:calcFeatures>
+        <ns9:feature name="microsoft.com:RD"/>
+        <ns9:feature name="microsoft.com:Single"/>
+        <ns9:feature name="microsoft.com:FV"/>
+        <ns9:feature name="microsoft.com:CNMTM"/>
+        <ns9:feature name="microsoft.com:LET_WF"/>
+        <ns9:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns9:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns9:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1704,6 +1705,641 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac xr xr2 xr3" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}"><dimension ref="A2:F61"/><sheetFormatPr baseColWidth="10" defaultRowHeight="15"/><cols><col min="1" max="1" width="6.5703125" customWidth="1"/><col min="2" max="2" width="23.7109375" customWidth="1"/><col min="3" max="3" width="15" customWidth="1"/><col min="4" max="4" width="5.7109375" customWidth="1"/><col min="5" max="5" width="11.28515625" customWidth="1"/><col min="6" max="6" width="16.85546875" customWidth="1"/></cols><sheetData><row r="2" spans="1:6" ht="22.5" customHeight="1"><c r="F2" s="7"/></row><row r="3" spans="1:6"><c r="F3" s="2"/></row><row r="4" spans="1:6"><c r="E4" s="20"/><c r="F4" s="4"/></row><row r="5" spans="1:6"><c r="E5" s="20" t="s"><v>1</v></c><c r="F5" s="4"></c></row><row r="6" spans="1:6" ht="16.5"><c r="A6" s="1" t="s"><v>0</v></c><c r="B6" s="1"/><c r="E6" s="5"/><c r="F6" s="5"/></row><row r="7" spans="1:6"><c r="E7" s="20"/><c r="F7" s="3"></c></row><row r="8" spans="1:6"><c r="E8" s="3"/><c r="F8" s="3"></c></row><row r="9" spans="1:6"><c r="E9" s="5"/><c r="F9" s="3"></c></row><row r="10" spans="1:6"><c r="E10" s="5"/><c r="F10" s="3"></c></row><row r="12" spans="1:6" ht="7.5" customHeight="1"/><row r="14" spans="1:6"><c r="A14" s="5" t="s"><v>3</v></c><c r="B14" s="5" t="s"><v>4</v></c><c r="C14" s="25" t="s"><v>6</v></c><c r="D14" s="25" t="s"><v>5</v></c></row><row r="15" spans="1:6" hidden="1"><c r="A15" s="26"><v>0</v></c><c r="B15" s="21" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C15" s="22" t="s"><v>8</v></c><c r="D15" s="23" t="s"><v>15</v></c></row><row r="16" spans="1:6" hidden="1"><c r="A16" s="27"><v>0</v></c><c r="B16" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C16" s="16" t="s"><v>8</v></c><c r="D16" s="14" t="s"><v>16</v></c></row><row r="17" spans="1:4"><c r="A17" s="27"><v>18</v></c><c r="B17" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C17" s="16" t="s"><v>8</v></c><c r="D17" s="14" t="s"><v>17</v></c></row><row r="18" spans="1:4" hidden="1"><c r="A18" s="27"><v>0</v></c><c r="B18" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C18" s="16" t="s"><v>11</v></c><c r="D18" s="14" t="s"><v>15</v></c></row><row r="19" spans="1:4" hidden="1"><c r="A19" s="27"><v>0</v></c><c r="B19" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C19" s="16" t="s"><v>11</v></c><c r="D19" s="14" t="s"><v>16</v></c></row><row r="20" spans="1:4" hidden="1"><c r="A20" s="27"><v>0</v></c><c r="B20" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C20" s="16" t="s"><v>11</v></c><c r="D20" s="14" t="s"><v>17</v></c></row><row r="21" spans="1:4" hidden="1"><c r="A21" s="27"><v>0</v></c><c r="B21" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C21" s="16" t="s"><v>9</v></c><c r="D21" s="14" t="s"><v>15</v></c></row><row r="22" spans="1:4" hidden="1"><c r="A22" s="27"><v>0</v></c><c r="B22" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C22" s="16" t="s"><v>9</v></c><c r="D22" s="14" t="s"><v>16</v></c></row><row r="23" spans="1:4" hidden="1"><c r="A23" s="27"><v>0</v></c><c r="B23" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C23" s="16" t="s"><v>9</v></c><c r="D23" s="14" t="s"><v>17</v></c></row><row r="24" spans="1:4" hidden="1"><c r="A24" s="27"><v>0</v></c><c r="B24" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C24" s="16" t="s"><v>10</v></c><c r="D24" s="14" t="s"><v>15</v></c></row><row r="25" spans="1:4" hidden="1"><c r="A25" s="27"><v>0</v></c><c r="B25" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C25" s="16" t="s"><v>10</v></c><c r="D25" s="14" t="s"><v>16</v></c></row><row r="26" spans="1:4" hidden="1"><c r="A26" s="27"><v>0</v></c><c r="B26" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C26" s="16" t="s"><v>10</v></c><c r="D26" s="14" t="s"><v>17</v></c></row><row r="27" spans="1:4" hidden="1"><c r="A27" s="27"><v>0</v></c><c r="B27" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C27" s="16" t="s"><v>12</v></c><c r="D27" s="14" t="s"><v>15</v></c></row><row r="28" spans="1:4" hidden="1"><c r="A28" s="27"><v>0</v></c><c r="B28" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C28" s="16" t="s"><v>12</v></c><c r="D28" s="14" t="s"><v>16</v></c></row><row r="29" spans="1:4"><c r="A29" s="27"><v>6</v></c><c r="B29" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C29" s="16" t="s"><v>12</v></c><c r="D29" s="15" t="s"><v>17</v></c></row><row r="30" spans="1:4" hidden="1"><c r="A30" s="27"><v>0</v></c><c r="B30" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C30" s="16" t="s"><v>91</v></c><c r="D30" s="15" t="s"><v>15</v></c></row><row r="31" spans="1:4" hidden="1"><c r="A31" s="27"><v>0</v></c><c r="B31" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C31" s="16" t="s"><v>91</v></c><c r="D31" s="15" t="s"><v>16</v></c></row><row r="32" spans="1:4"><c r="A32" s="27"><v>24</v></c><c r="B32" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C32" s="16" t="s"><v>91</v></c><c r="D32" s="15" t="s"><v>17</v></c></row><row r="33" spans="1:5" hidden="1"><c r="A33" s="27"><v>0</v></c><c r="B33" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C33" s="16" t="s"><v>203</v></c><c r="D33" s="15" t="s"><v>15</v></c></row><row r="34" spans="1:5" hidden="1"><c r="A34" s="27"><v>0</v></c><c r="B34" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C34" s="16" t="s"><v>203</v></c><c r="D34" s="15" t="s"><v>16</v></c></row><row r="35" spans="1:5"><c r="A35" s="27"><v>12</v></c><c r="B35" s="39" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v>ThéCol - Thé Froid Artisanal</v></c><c r="C35" s="16" t="s"><v>203</v></c><c r="D35" s="15" t="s"><v>17</v></c></row><row r="36" spans="1:5" hidden="1"><c r="A36" s="27"><v>0</v></c><c r="B36" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C36" s="16" t="s"><v>13</v></c><c r="D36" s="14" t="s"><v>15</v></c></row><row r="37" spans="1:5" hidden="1"><c r="A37" s="27"><v>0</v></c><c r="B37" s="10" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C37" s="17" t="s"><v>13</v></c><c r="D37" s="14" t="s"><v>16</v></c></row><row r="38" spans="1:5" hidden="1"><c r="A38" s="27"><v>0</v></c><c r="B38" s="24" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C38" s="16" t="s"><v>13</v></c><c r="D38" s="15" t="s"><v>17</v></c></row><row r="39" spans="1:5" ht="14.25" customHeight="1"><c r="A39" s="27"/><c r="B39" s="10"/><c r="C39" s="13"/><c r="D39" s="11"/></row><row r="40" spans="1:5" ht="14.25" customHeight="1"><c r="A40" s="30"/><c r="B40" s="12"/><c r="C40" s="5"/><c r="D40" s="5"/></row><row r="41" spans="1:5" ht="2.25" hidden="1" customHeight="1"><c r="A41" s="27"><v>0</v></c><c r="B41" s="10" t="s"><v>92</v></c><c r="C41" s="11"/><c r="D41" s="31"/></row><row r="42" spans="1:5" hidden="1"><c r="A42" s="27"><v>0</v></c><c r="B42" s="10" t="s"><v>92</v></c><c r="C42" s="12"/><c r="D42" s="11"/></row><row r="43" spans="1:5" hidden="1"><c r="A43" s="27"><v>0</v></c><c r="B43" s="10" t="s"><v>90</v></c><c r="C43" s="13" t="s"><v>95</v></c><c r="D43" s="11" t="s"><v>17</v></c></row><row r="44" spans="1:5"><c r="A44" s="5"/><c r="B44" s="5" t="str"><f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f><v xml:space="preserve"> </v></c><c r="C44" s="5"/><c r="D44" s="5"/></row><row r="45" spans="1:5" ht="14.25" customHeight="1"/><row r="46" spans="1:5" ht="15" customHeight="1"><c r="B46" s="19"/><c r="C46" s="18"/><c r="D46" t="s"><v>204</v></c></row><row r="47" spans="1:5" ht="15" customHeight="1" thickBot="1"><c r="B47" s="18"/><c r="C47" s="18"/><c r="D47" s="2"></c><c r="E47" t="s"><v>96</v></c></row><row r="48" spans="1:5" ht="15" customHeight="1" thickBot="1"><c r="A48" s="32"><v>0</v></c><c r="B48" s="28" t="s"><v>79</v></c><c r="C48" s="18"/><c r="D48" s="2"></c><c r="E48" t="s"><v>97</v></c></row><row r="49" spans="1:6" ht="15" customHeight="1" thickBot="1"><c r="A49" s="32"><v>3</v></c><c r="B49" s="28" t="s"><v>80</v></c><c r="C49" s="18"/><c r="D49" s="2"></c><c r="E49" s="36" t="s"><v>93</v></c></row><row r="50" spans="1:6" ht="15" customHeight="1" thickBot="1"><c r="A50" s="32"/><c r="B50" s="28" t="s"><v>81</v></c><c r="C50" s="18"/><c r="D50" s="2"/></row><row r="51" spans="1:6" ht="15.75" thickBot="1"><c r="A51" s="34"/><c r="B51" s="28" t="s"><v>82</v></c><c r="C51" s="18"/><c r="D51" t="s"><v>98</v></c><c r="E51" s="40"></c><c r="F51" s="2"/></row><row r="52" spans="1:6" ht="28.5" customHeight="1"><c r="B52" s="28"/><c r="C52" s="18"/><c r="E52" s="2"/><c r="F52" s="2"/></row><row r="53" spans="1:6"><c r="B53" s="18"/><c r="C53" s="18"/><c r="E53" s="2"/><c r="F53" s="2"/></row><row r="54" spans="1:6" ht="21"><c r="A54" s="6"></c><c r="B54" s="18"/><c r="C54" s="18"/><c r="E54" s="2"/><c r="F54" s="2"/></row><row r="55" spans="1:6" ht="42" customHeight="1"><c r="E55" s="2"/><c r="F55" s="2"/></row><row r="56" spans="1:6" ht="21"><c r="A56" s="6" t="s"><v>2</v></c><c r="B56" s="6"/><c r="E56" s="2"/><c r="F56" s="2"/></row><row r="57" spans="1:6" ht="51" customHeight="1"><c r="D57" s="38" t="e" vm="1"><v>#VALUE!</v></c><c r="E57" s="38"/><c r="F57" s="38"/></row><row r="58" spans="1:6"><c r="B58" s="38"/><c r="D58" s="38"/><c r="E58" s="38"/><c r="F58" s="38"/></row><row r="59" spans="1:6"><c r="B59" s="38"/><c r="D59" s="38"/><c r="E59" s="38"/><c r="F59" s="38"/></row><row r="60" spans="1:6"><c r="D60" s="2"/></row><row r="61" spans="1:6"><c r="D61" s="2"/></row></sheetData><mergeCells count="2"><mergeCell ref="B58:B59"/><mergeCell ref="D57:F59"/></mergeCells><pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/><pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/><drawing r:id="rId2"/><tableParts count="1"><tablePart r:id="rId3"/></tableParts><extLst><ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main"></x14:dataValidations></ext></extLst></worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
+  <dimension ref="A2:F61"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="6.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" ht="22.5" customHeight="1">
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="E4" s="20"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="E5" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" ht="16.5">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="E7" s="20"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="E9" s="5"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="E10" s="5"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="12" spans="1:6" ht="7.5" customHeight="1"/>
+    <row r="14" spans="1:6">
+      <c r="A14" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" hidden="1">
+      <c r="A15" s="26">
+        <v>0</v>
+      </c>
+      <c r="B15" s="21" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" hidden="1">
+      <c r="A16" s="27">
+        <v>0</v>
+      </c>
+      <c r="B16" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="27">
+        <v>18</v>
+      </c>
+      <c r="B17" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v>ThéCol - Thé Froid Artisanal</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" hidden="1">
+      <c r="A18" s="27">
+        <v>0</v>
+      </c>
+      <c r="B18" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" hidden="1">
+      <c r="A19" s="27">
+        <v>0</v>
+      </c>
+      <c r="B19" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" hidden="1">
+      <c r="A20" s="27">
+        <v>0</v>
+      </c>
+      <c r="B20" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" hidden="1">
+      <c r="A21" s="27">
+        <v>0</v>
+      </c>
+      <c r="B21" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" hidden="1">
+      <c r="A22" s="27">
+        <v>0</v>
+      </c>
+      <c r="B22" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" hidden="1">
+      <c r="A23" s="27">
+        <v>0</v>
+      </c>
+      <c r="B23" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" hidden="1">
+      <c r="A24" s="27">
+        <v>0</v>
+      </c>
+      <c r="B24" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" hidden="1">
+      <c r="A25" s="27">
+        <v>0</v>
+      </c>
+      <c r="B25" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" hidden="1">
+      <c r="A26" s="27">
+        <v>0</v>
+      </c>
+      <c r="B26" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" hidden="1">
+      <c r="A27" s="27">
+        <v>0</v>
+      </c>
+      <c r="B27" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" hidden="1">
+      <c r="A28" s="27">
+        <v>0</v>
+      </c>
+      <c r="B28" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="27">
+        <v>6</v>
+      </c>
+      <c r="B29" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v>ThéCol - Thé Froid Artisanal</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" hidden="1">
+      <c r="A30" s="27">
+        <v>0</v>
+      </c>
+      <c r="B30" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" hidden="1">
+      <c r="A31" s="27">
+        <v>0</v>
+      </c>
+      <c r="B31" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="27">
+        <v>24</v>
+      </c>
+      <c r="B32" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v>ThéCol - Thé Froid Artisanal</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" hidden="1">
+      <c r="A33" s="27">
+        <v>0</v>
+      </c>
+      <c r="B33" s="39" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" hidden="1">
+      <c r="A34" s="27">
+        <v>0</v>
+      </c>
+      <c r="B34" s="39" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="27">
+        <v>12</v>
+      </c>
+      <c r="B35" s="39" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v>ThéCol - Thé Froid Artisanal</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" hidden="1">
+      <c r="A36" s="27">
+        <v>0</v>
+      </c>
+      <c r="B36" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" hidden="1">
+      <c r="A37" s="27">
+        <v>0</v>
+      </c>
+      <c r="B37" s="10" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" hidden="1">
+      <c r="A38" s="27">
+        <v>0</v>
+      </c>
+      <c r="B38" s="24" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A39" s="27"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="11"/>
+    </row>
+    <row r="40" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A40" s="30"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+    </row>
+    <row r="41" spans="1:5" ht="2.25" hidden="1" customHeight="1">
+      <c r="A41" s="27">
+        <v>0</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="11"/>
+      <c r="D41" s="31"/>
+    </row>
+    <row r="42" spans="1:5" hidden="1">
+      <c r="A42" s="27">
+        <v>0</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42" s="12"/>
+      <c r="D42" s="11"/>
+    </row>
+    <row r="43" spans="1:5" hidden="1">
+      <c r="A43" s="27">
+        <v>0</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="str">
+        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+    </row>
+    <row r="45" spans="1:5" ht="14.25" customHeight="1"/>
+    <row r="46" spans="1:5" ht="15" customHeight="1">
+      <c r="B46" s="19"/>
+      <c r="C46" s="18"/>
+      <c r="D46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="2"/>
+      <c r="E47" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15" customHeight="1" thickBot="1">
+      <c r="A48" s="32">
+        <v>0</v>
+      </c>
+      <c r="B48" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C48" s="18"/>
+      <c r="D48" s="2"/>
+      <c r="E48" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="15" customHeight="1" thickBot="1">
+      <c r="A49" s="32">
+        <v>3</v>
+      </c>
+      <c r="B49" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="18"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="36" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="15" customHeight="1" thickBot="1">
+      <c r="A50" s="32"/>
+      <c r="B50" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="C50" s="18"/>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="1:6" ht="15.75" thickBot="1">
+      <c r="A51" s="34"/>
+      <c r="B51" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" s="18"/>
+      <c r="D51" t="s">
+        <v>98</v>
+      </c>
+      <c r="E51" s="40"/>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" spans="1:6" ht="28.5" customHeight="1">
+      <c r="B52" s="28"/>
+      <c r="C52" s="18"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+    </row>
+    <row r="54" spans="1:6" ht="21">
+      <c r="A54" s="6"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" spans="1:6" ht="42" customHeight="1">
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="1:6" ht="21">
+      <c r="A56" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+    </row>
+    <row r="57" spans="1:6" ht="51" customHeight="1">
+      <c r="D57" s="38" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="B58" s="38"/>
+      <c r="D58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38"/>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="B59" s="38"/>
+      <c r="D59" s="38"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38"/>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="D60" s="2"/>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="D61" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="D57:F59"/>
+  </mergeCells>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
+  <extLst>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns4:dataValidations count="3">
+        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F88F0296-B037-4558-8BF3-BF1788835FEC}">
+          <ns4:formula1>
+            <ns5:f>'Listes '!$E:$E</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>F7</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F91DE666-C1EC-46FF-BFAC-77ABE88F7950}">
+          <ns4:formula1>
+            <ns5:f>'Listes '!$A$2:$A$13</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>C15:C38</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B9B91086-C40D-46C4-8549-1E3A0C7DF361}">
+          <ns4:formula1>
+            <ns5:f>'Listes '!$B$2:$B$13</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>D15:D38</ns5:sqref>
+        </ns4:dataValidation>
+      </ns4:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Hotfix: clean extLst namespace prefixes, fix D57 error cell, bump v5.8
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -2282,9 +2282,7 @@
       <c r="F56" s="2"/>
     </row>
     <row r="57" spans="1:6" ht="51" customHeight="1">
-      <c r="D57" s="38" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="D57" s="38"/>
       <c r="E57" s="38"/>
       <c r="F57" s="38"/>
     </row>
@@ -2318,28 +2316,7 @@
     <tablePart r:id="rId3"/>
   </tableParts>
   <extLst>
-    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <ns4:dataValidations count="3">
-        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F88F0296-B037-4558-8BF3-BF1788835FEC}">
-          <ns4:formula1>
-            <ns5:f>'Listes '!$E:$E</ns5:f>
-          </ns4:formula1>
-          <ns5:sqref>F7</ns5:sqref>
-        </ns4:dataValidation>
-        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F91DE666-C1EC-46FF-BFAC-77ABE88F7950}">
-          <ns4:formula1>
-            <ns5:f>'Listes '!$A$2:$A$13</ns5:f>
-          </ns4:formula1>
-          <ns5:sqref>C15:C38</ns5:sqref>
-        </ns4:dataValidation>
-        <ns4:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B9B91086-C40D-46C4-8549-1E3A0C7DF361}">
-          <ns4:formula1>
-            <ns5:f>'Listes '!$B$2:$B$13</ns5:f>
-          </ns4:formula1>
-          <ns5:sqref>D15:D38</ns5:sqref>
-        </ns4:dataValidation>
-      </ns4:dataValidations>
-    </ext>
+    <ext uri="{CCE6A557-97BC-4B89-ADB6-D9C93CAAB3DF}"/>
   </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Hotfix: rebuild bl_template.xlsx with correct Content_Types/references, clean cells, v5.9
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -1,36 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <ns2:absPath url="C:\Users\noahb\Desktop\Thécol\Finances\Livraison et facturation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahb\Desktop\Thécol\Finances\Livraison et facturation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF0E999-4ECE-4970-AD15-5307EE881E75}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF0E999-4ECE-4970-AD15-5307EE881E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2085" windowWidth="28800" windowHeight="15345" xr2:uid="{C5804516-DE8A-4579-A9F8-8DDE14F0BC4E}"/>
   </bookViews>
-  <sheets>
-    <sheet name="Bulletin de livraison" sheetId="1" r:id="rId1"/>
-    <sheet name="Listes " sheetId="2" r:id="rId2"/>
-  </sheets>
+  <sheets/>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <ns8:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <ns9:calcFeatures>
-        <ns9:feature name="microsoft.com:RD"/>
-        <ns9:feature name="microsoft.com:Single"/>
-        <ns9:feature name="microsoft.com:FV"/>
-        <ns9:feature name="microsoft.com:CNMTM"/>
-        <ns9:feature name="microsoft.com:LET_WF"/>
-        <ns9:feature name="microsoft.com:LAMBDA_WF"/>
-        <ns9:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </ns9:calcFeatures>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1706,7 +1703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
   <dimension ref="A2:F61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
@@ -2315,8 +2312,5 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
-  <extLst>
-    <ext uri="{CCE6A557-97BC-4B89-ADB6-D9C93CAAB3DF}"/>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Robustness pass: harden DB/modal/toast/render with null checks, validation, try/catch; rebuild clean bl_template.xlsx from original, v5.14
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -12,7 +12,9 @@
   <bookViews>
     <workbookView xWindow="3660" yWindow="2085" windowWidth="28800" windowHeight="15345" xr2:uid="{C5804516-DE8A-4579-A9F8-8DDE14F0BC4E}"/>
   </bookViews>
-  <sheets/>
+  <sheets>
+    <sheet name="Bulletin de livraison" sheetId="1" r:id="rId1"/>
+  </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1703,7 +1705,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
   <dimension ref="A2:F61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
@@ -1729,7 +1731,10 @@
       <c r="E5" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="4">
+        <f ca="1">TODAY()</f>
+        <v>45953</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="16.5">
       <c r="A6" s="1" t="s">
@@ -1741,19 +1746,30 @@
     </row>
     <row r="7" spans="1:6">
       <c r="E7" s="20"/>
-      <c r="F7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3" t="str">
+        <f>VLOOKUP(F7,Tableau4[],2,FALSE)</f>
+        <v xml:space="preserve">Ines Haymoz </v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="E9" s="5"/>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3" t="str">
+        <f>VLOOKUP(F7,Tableau4[],3,FALSE)</f>
+        <v>Derrière-les-Jardins 2</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
       <c r="E10" s="5"/>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3" t="str">
+        <f>VLOOKUP(F7,Tableau4[],4,FALSE)</f>
+        <v>1700 Fribourg</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="7.5" customHeight="1"/>
     <row r="14" spans="1:6">
@@ -2196,7 +2212,10 @@
     <row r="47" spans="1:5" ht="15" customHeight="1" thickBot="1">
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
-      <c r="D47" s="2"/>
+      <c r="D47" s="2" t="str">
+        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="E-Mail","x"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
       <c r="E47" t="s">
         <v>96</v>
       </c>
@@ -2209,7 +2228,10 @@
         <v>79</v>
       </c>
       <c r="C48" s="18"/>
-      <c r="D48" s="2"/>
+      <c r="D48" s="2" t="str">
+        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="Envoi postal","x"," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
       <c r="E48" t="s">
         <v>97</v>
       </c>
@@ -2222,7 +2244,10 @@
         <v>80</v>
       </c>
       <c r="C49" s="18"/>
-      <c r="D49" s="2"/>
+      <c r="D49" s="2" t="str">
+        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="Autre","x"," ")</f>
+        <v>x</v>
+      </c>
       <c r="E49" s="36" t="s">
         <v>93</v>
       </c>
@@ -2244,7 +2269,10 @@
       <c r="D51" t="s">
         <v>98</v>
       </c>
-      <c r="E51" s="40"/>
+      <c r="E51" s="40" t="str">
+        <f>VLOOKUP(F7,Tableau4[],10,FALSE)</f>
+        <v>sur place à la livraison</v>
+      </c>
       <c r="F51" s="2"/>
     </row>
     <row r="52" spans="1:6" ht="28.5" customHeight="1">
@@ -2260,7 +2288,10 @@
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="1:6" ht="21">
-      <c r="A54" s="6"/>
+      <c r="A54" s="6" t="str">
+        <f>F7</f>
+        <v>Café de la Marionnette</v>
+      </c>
       <c r="B54" s="18"/>
       <c r="C54" s="18"/>
       <c r="E54" s="2"/>
@@ -2279,7 +2310,9 @@
       <c r="F56" s="2"/>
     </row>
     <row r="57" spans="1:6" ht="51" customHeight="1">
-      <c r="D57" s="38"/>
+      <c r="D57" s="38" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="E57" s="38"/>
       <c r="F57" s="38"/>
     </row>
@@ -2312,5 +2345,29 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F88F0296-B037-4558-8BF3-BF1788835FEC}">
+          <x14:formula1>
+            <xm:f>'Listes '!$E:$E</xm:f>
+          </x14:formula1>
+          <xm:sqref>F7</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F91DE666-C1EC-46FF-BFAC-77ABE88F7950}">
+          <x14:formula1>
+            <xm:f>'Listes '!$A$2:$A$13</xm:f>
+          </x14:formula1>
+          <xm:sqref>C15:C38</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B9B91086-C40D-46C4-8549-1E3A0C7DF361}">
+          <x14:formula1>
+            <xm:f>'Listes '!$B$2:$B$13</xm:f>
+          </x14:formula1>
+          <xm:sqref>D15:D38</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix BL export: strip all formulas/extLst from template, force cell overwrite on empty data, add XML declaration, v5.15
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -1732,7 +1732,6 @@
         <v>1</v>
       </c>
       <c r="F5" s="4">
-        <f ca="1">TODAY()</f>
         <v>45953</v>
       </c>
     </row>
@@ -1753,21 +1752,18 @@
     <row r="8" spans="1:6">
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="str">
-        <f>VLOOKUP(F7,Tableau4[],2,FALSE)</f>
         <v xml:space="preserve">Ines Haymoz </v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="E9" s="5"/>
       <c r="F9" s="3" t="str">
-        <f>VLOOKUP(F7,Tableau4[],3,FALSE)</f>
         <v>Derrière-les-Jardins 2</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="E10" s="5"/>
       <c r="F10" s="3" t="str">
-        <f>VLOOKUP(F7,Tableau4[],4,FALSE)</f>
         <v>1700 Fribourg</v>
       </c>
     </row>
@@ -1791,7 +1787,6 @@
         <v>0</v>
       </c>
       <c r="B15" s="21" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C15" s="22" t="s">
@@ -1806,7 +1801,6 @@
         <v>0</v>
       </c>
       <c r="B16" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C16" s="16" t="s">
@@ -1821,7 +1815,6 @@
         <v>18</v>
       </c>
       <c r="B17" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v>ThéCol - Thé Froid Artisanal</v>
       </c>
       <c r="C17" s="16" t="s">
@@ -1836,7 +1829,6 @@
         <v>0</v>
       </c>
       <c r="B18" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C18" s="16" t="s">
@@ -1851,7 +1843,6 @@
         <v>0</v>
       </c>
       <c r="B19" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C19" s="16" t="s">
@@ -1866,7 +1857,6 @@
         <v>0</v>
       </c>
       <c r="B20" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C20" s="16" t="s">
@@ -1881,7 +1871,6 @@
         <v>0</v>
       </c>
       <c r="B21" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C21" s="16" t="s">
@@ -1896,7 +1885,6 @@
         <v>0</v>
       </c>
       <c r="B22" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C22" s="16" t="s">
@@ -1911,7 +1899,6 @@
         <v>0</v>
       </c>
       <c r="B23" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C23" s="16" t="s">
@@ -1926,7 +1913,6 @@
         <v>0</v>
       </c>
       <c r="B24" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C24" s="16" t="s">
@@ -1941,7 +1927,6 @@
         <v>0</v>
       </c>
       <c r="B25" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C25" s="16" t="s">
@@ -1956,7 +1941,6 @@
         <v>0</v>
       </c>
       <c r="B26" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C26" s="16" t="s">
@@ -1971,7 +1955,6 @@
         <v>0</v>
       </c>
       <c r="B27" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C27" s="16" t="s">
@@ -1986,7 +1969,6 @@
         <v>0</v>
       </c>
       <c r="B28" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C28" s="16" t="s">
@@ -2001,7 +1983,6 @@
         <v>6</v>
       </c>
       <c r="B29" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v>ThéCol - Thé Froid Artisanal</v>
       </c>
       <c r="C29" s="16" t="s">
@@ -2016,7 +1997,6 @@
         <v>0</v>
       </c>
       <c r="B30" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C30" s="16" t="s">
@@ -2031,7 +2011,6 @@
         <v>0</v>
       </c>
       <c r="B31" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C31" s="16" t="s">
@@ -2046,7 +2025,6 @@
         <v>24</v>
       </c>
       <c r="B32" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v>ThéCol - Thé Froid Artisanal</v>
       </c>
       <c r="C32" s="16" t="s">
@@ -2061,7 +2039,6 @@
         <v>0</v>
       </c>
       <c r="B33" s="39" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C33" s="16" t="s">
@@ -2076,7 +2053,6 @@
         <v>0</v>
       </c>
       <c r="B34" s="39" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C34" s="16" t="s">
@@ -2091,7 +2067,6 @@
         <v>12</v>
       </c>
       <c r="B35" s="39" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v>ThéCol - Thé Froid Artisanal</v>
       </c>
       <c r="C35" s="16" t="s">
@@ -2106,7 +2081,6 @@
         <v>0</v>
       </c>
       <c r="B36" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C36" s="16" t="s">
@@ -2121,7 +2095,6 @@
         <v>0</v>
       </c>
       <c r="B37" s="10" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C37" s="17" t="s">
@@ -2136,7 +2109,6 @@
         <v>0</v>
       </c>
       <c r="B38" s="24" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C38" s="16" t="s">
@@ -2195,7 +2167,6 @@
     <row r="44" spans="1:5">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="str">
-        <f>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="C44" s="5"/>
@@ -2213,7 +2184,6 @@
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
       <c r="D47" s="2" t="str">
-        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="E-Mail","x"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="E47" t="s">
@@ -2229,7 +2199,6 @@
       </c>
       <c r="C48" s="18"/>
       <c r="D48" s="2" t="str">
-        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="Envoi postal","x"," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="E48" t="s">
@@ -2245,7 +2214,6 @@
       </c>
       <c r="C49" s="18"/>
       <c r="D49" s="2" t="str">
-        <f>IF(VLOOKUP(F7,Tableau4[],9,FALSE)="Autre","x"," ")</f>
         <v>x</v>
       </c>
       <c r="E49" s="36" t="s">
@@ -2270,7 +2238,6 @@
         <v>98</v>
       </c>
       <c r="E51" s="40" t="str">
-        <f>VLOOKUP(F7,Tableau4[],10,FALSE)</f>
         <v>sur place à la livraison</v>
       </c>
       <c r="F51" s="2"/>
@@ -2289,7 +2256,6 @@
     </row>
     <row r="54" spans="1:6" ht="21">
       <c r="A54" s="6" t="str">
-        <f>F7</f>
         <v>Café de la Marionnette</v>
       </c>
       <c r="B54" s="18"/>
@@ -2345,29 +2311,5 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F88F0296-B037-4558-8BF3-BF1788835FEC}">
-          <x14:formula1>
-            <xm:f>'Listes '!$E:$E</xm:f>
-          </x14:formula1>
-          <xm:sqref>F7</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F91DE666-C1EC-46FF-BFAC-77ABE88F7950}">
-          <x14:formula1>
-            <xm:f>'Listes '!$A$2:$A$13</xm:f>
-          </x14:formula1>
-          <xm:sqref>C15:C38</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B9B91086-C40D-46C4-8549-1E3A0C7DF361}">
-          <x14:formula1>
-            <xm:f>'Listes '!$B$2:$B$13</xm:f>
-          </x14:formula1>
-          <xm:sqref>D15:D38</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix BL export: prevent double XML declaration, inject ThéCol desc in col B, v5.16
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -1379,9 +1379,7 @@
   </autoFilter>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{1A477314-2E09-4C98-BAC6-896516FACBCF}" name="QTT" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{38558BE9-82AC-43AB-A07D-B067A83EA99E}" name="Description" dataDxfId="7">
-      <calculatedColumnFormula>IF(Tableau1[[#This Row],[QTT]]&lt;&gt;0,"ThéCol - Thé Froid Artisanal"," ")</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="2" xr3:uid="{38558BE9-82AC-43AB-A07D-B067A83EA99E}" name="Description" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{8422D6DD-456B-478D-A22C-DE624EDE619C}" name="Arôme" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{975D51B1-3BEB-45A8-9486-4C2BEDCCBA24}" name="Format" dataDxfId="5"/>
   </tableColumns>

</xml_diff>

<commit_message>
fix: renforcer sécurité, sync et export BL v11.6
</commit_message>
<xml_diff>
--- a/templates/bl_template.xlsx
+++ b/templates/bl_template.xlsx
@@ -664,7 +664,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 4" descr="Une image contenant texte&#10;&#10;Description générée automatiquement">
+        <xdr:cNvPr id="5" name="Image 4" descr="Une image contenant texte Description générée automatiquement">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{680B099F-F326-9EE0-6C45-94DD39D8BBE7}"/>
@@ -1220,7 +1220,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333C3373-AE42-4256-BB11-C40A43E6AE39}">
   <dimension ref="A2:F61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
@@ -1301,336 +1301,336 @@
       <c r="A15" s="24">
         <v>0</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>13</v>
+      <c r="B15" s="19">
+        <v>0</v>
+      </c>
+      <c r="C15" s="20">
+        <v>0</v>
+      </c>
+      <c r="D15" s="21">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" hidden="1">
       <c r="A16" s="25">
         <v>0</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="B16" s="8">
+        <v>0</v>
+      </c>
+      <c r="C16" s="14">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" hidden="1">
       <c r="A17" s="25">
-        <v>18</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0</v>
+      </c>
+      <c r="C17" s="14">
+        <v>0</v>
+      </c>
+      <c r="D17" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:4" hidden="1">
       <c r="A18" s="25">
         <v>0</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>13</v>
+      <c r="B18" s="8">
+        <v>0</v>
+      </c>
+      <c r="C18" s="14">
+        <v>0</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:4" hidden="1">
       <c r="A19" s="25">
         <v>0</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>14</v>
+      <c r="B19" s="8">
+        <v>0</v>
+      </c>
+      <c r="C19" s="14">
+        <v>0</v>
+      </c>
+      <c r="D19" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:4" hidden="1">
       <c r="A20" s="25">
         <v>0</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>15</v>
+      <c r="B20" s="8">
+        <v>0</v>
+      </c>
+      <c r="C20" s="14">
+        <v>0</v>
+      </c>
+      <c r="D20" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" hidden="1">
       <c r="A21" s="25">
         <v>0</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>13</v>
+      <c r="B21" s="8">
+        <v>0</v>
+      </c>
+      <c r="C21" s="14">
+        <v>0</v>
+      </c>
+      <c r="D21" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:4" hidden="1">
       <c r="A22" s="25">
         <v>0</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>14</v>
+      <c r="B22" s="8">
+        <v>0</v>
+      </c>
+      <c r="C22" s="14">
+        <v>0</v>
+      </c>
+      <c r="D22" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:4" hidden="1">
       <c r="A23" s="25">
         <v>0</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>15</v>
+      <c r="B23" s="8">
+        <v>0</v>
+      </c>
+      <c r="C23" s="14">
+        <v>0</v>
+      </c>
+      <c r="D23" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:4" hidden="1">
       <c r="A24" s="25">
         <v>0</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>13</v>
+      <c r="B24" s="8">
+        <v>0</v>
+      </c>
+      <c r="C24" s="14">
+        <v>0</v>
+      </c>
+      <c r="D24" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:4" hidden="1">
       <c r="A25" s="25">
         <v>0</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>14</v>
+      <c r="B25" s="8">
+        <v>0</v>
+      </c>
+      <c r="C25" s="14">
+        <v>0</v>
+      </c>
+      <c r="D25" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4" hidden="1">
       <c r="A26" s="25">
         <v>0</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>15</v>
+      <c r="B26" s="8">
+        <v>0</v>
+      </c>
+      <c r="C26" s="14">
+        <v>0</v>
+      </c>
+      <c r="D26" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4" hidden="1">
       <c r="A27" s="25">
         <v>0</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>13</v>
+      <c r="B27" s="8">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14">
+        <v>0</v>
+      </c>
+      <c r="D27" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:4" hidden="1">
       <c r="A28" s="25">
         <v>0</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="B28" s="8">
+        <v>0</v>
+      </c>
+      <c r="C28" s="14">
+        <v>0</v>
+      </c>
+      <c r="D28" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" hidden="1">
       <c r="A29" s="25">
-        <v>6</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="B29" s="8">
+        <v>0</v>
+      </c>
+      <c r="C29" s="14">
+        <v>0</v>
+      </c>
+      <c r="D29" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:4" hidden="1">
       <c r="A30" s="25">
         <v>0</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>13</v>
+      <c r="B30" s="8">
+        <v>0</v>
+      </c>
+      <c r="C30" s="14">
+        <v>0</v>
+      </c>
+      <c r="D30" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:4" hidden="1">
       <c r="A31" s="25">
         <v>0</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="B31" s="8">
+        <v>0</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
+      </c>
+      <c r="D31" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" hidden="1">
       <c r="A32" s="25">
-        <v>24</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="B32" s="8">
+        <v>0</v>
+      </c>
+      <c r="C32" s="14">
+        <v>0</v>
+      </c>
+      <c r="D32" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5" hidden="1">
       <c r="A33" s="25">
         <v>0</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>13</v>
+      <c r="B33" s="8">
+        <v>0</v>
+      </c>
+      <c r="C33" s="14">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5" hidden="1">
       <c r="A34" s="25">
         <v>0</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="B34" s="8">
+        <v>0</v>
+      </c>
+      <c r="C34" s="14">
+        <v>0</v>
+      </c>
+      <c r="D34" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" hidden="1">
       <c r="A35" s="25">
-        <v>12</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="B35" s="8">
+        <v>0</v>
+      </c>
+      <c r="C35" s="14">
+        <v>0</v>
+      </c>
+      <c r="D35" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:5" hidden="1">
       <c r="A36" s="25">
         <v>0</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>13</v>
+      <c r="B36" s="8">
+        <v>0</v>
+      </c>
+      <c r="C36" s="14">
+        <v>0</v>
+      </c>
+      <c r="D36" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:5" hidden="1">
       <c r="A37" s="25">
         <v>0</v>
       </c>
-      <c r="B37" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>14</v>
+      <c r="B37" s="8">
+        <v>0</v>
+      </c>
+      <c r="C37" s="15">
+        <v>0</v>
+      </c>
+      <c r="D37" s="12">
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:5" hidden="1">
       <c r="A38" s="25">
         <v>0</v>
       </c>
-      <c r="B38" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>15</v>
+      <c r="B38" s="22">
+        <v>0</v>
+      </c>
+      <c r="C38" s="14">
+        <v>0</v>
+      </c>
+      <c r="D38" s="13">
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14.25" customHeight="1">

</xml_diff>